<commit_message>
detect unrecognized submit values
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ysyzy\code\day1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ysyzy\code\excel-merge-clean-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>姓名</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>王五</t>
+  </si>
+  <si>
+    <t>已交</t>
   </si>
 </sst>
 </file>
@@ -1244,7 +1247,7 @@
         <v>2026003</v>
       </c>
       <c r="C4" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
unify submit value rules and add web version
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="15160" windowHeight="9650"/>
+    <workbookView windowWidth="15380" windowHeight="10210"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
     <t>王五</t>
   </si>
   <si>
-    <t>已交</t>
+    <t>请假</t>
   </si>
 </sst>
 </file>

</xml_diff>